<commit_message>
Source Data: Fig. 2, Fig. 3 (own Ru/C bed series in panel d), ED Figs 4-5 on the corrected outputs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/SourceData_EDFig4.xlsx
+++ b/source_data/SourceData_EDFig4.xlsx
@@ -710,7 +710,7 @@
         <v>16641.02922668158</v>
       </c>
       <c r="H5" t="n">
-        <v>15.51555967209343</v>
+        <v>15.5091508671665</v>
       </c>
       <c r="J5" t="n">
         <v>157</v>
@@ -743,7 +743,7 @@
         <v>1920</v>
       </c>
       <c r="H6" t="n">
-        <v>15.5428780802548</v>
+        <v>15.54287801912185</v>
       </c>
       <c r="J6" t="n">
         <v>79</v>
@@ -776,7 +776,7 @@
         <v>12865.33351978744</v>
       </c>
       <c r="H7" t="n">
-        <v>15.68592688820667</v>
+        <v>15.68135157201682</v>
       </c>
       <c r="J7" t="n">
         <v>157</v>
@@ -809,10 +809,10 @@
         <v>604000</v>
       </c>
       <c r="H8" t="n">
-        <v>15.94026296255697</v>
+        <v>15.88075081788533</v>
       </c>
       <c r="I8" t="n">
-        <v>14.8011102438811</v>
+        <v>14.75844177235617</v>
       </c>
       <c r="J8" t="n">
         <v>106</v>
@@ -845,7 +845,7 @@
         <v>144000</v>
       </c>
       <c r="H9" t="n">
-        <v>16.01727564705142</v>
+        <v>16.01706713081194</v>
       </c>
       <c r="J9" t="n">
         <v>154</v>
@@ -878,10 +878,10 @@
         <v>158000</v>
       </c>
       <c r="H10" t="n">
-        <v>16.31299529741685</v>
+        <v>16.29624559873036</v>
       </c>
       <c r="I10" t="n">
-        <v>15.06886674201865</v>
+        <v>15.05550513764555</v>
       </c>
       <c r="J10" t="n">
         <v>116</v>
@@ -914,7 +914,7 @@
         <v>10875</v>
       </c>
       <c r="H11" t="n">
-        <v>16.31700896611387</v>
+        <v>16.31056913453592</v>
       </c>
       <c r="J11" t="n">
         <v>84</v>
@@ -980,10 +980,10 @@
         <v>3125000</v>
       </c>
       <c r="H13" t="n">
-        <v>17.52559198205939</v>
+        <v>17.22165142925473</v>
       </c>
       <c r="I13" t="n">
-        <v>15.59487250081747</v>
+        <v>15.49738797410795</v>
       </c>
       <c r="J13" t="n">
         <v>109</v>
@@ -1016,10 +1016,10 @@
         <v>105000</v>
       </c>
       <c r="H14" t="n">
-        <v>17.82126562995367</v>
+        <v>17.79478561142073</v>
       </c>
       <c r="I14" t="n">
-        <v>15.63295484288588</v>
+        <v>15.62490554740077</v>
       </c>
       <c r="J14" t="n">
         <v>105</v>
@@ -1052,7 +1052,7 @@
         <v>92307.6923076923</v>
       </c>
       <c r="H15" t="n">
-        <v>18.27959353487723</v>
+        <v>18.27631008120813</v>
       </c>
       <c r="J15" t="n">
         <v>199</v>
@@ -1085,7 +1085,7 @@
         <v>566666.6666666666</v>
       </c>
       <c r="H16" t="n">
-        <v>18.9240266858385</v>
+        <v>18.9237857349846</v>
       </c>
       <c r="J16" t="n">
         <v>82</v>
@@ -1118,10 +1118,10 @@
         <v>626000</v>
       </c>
       <c r="H17" t="n">
-        <v>19.26788699200953</v>
+        <v>19.22956838661794</v>
       </c>
       <c r="I17" t="n">
-        <v>16.48682528876611</v>
+        <v>16.46737343743095</v>
       </c>
       <c r="J17" t="n">
         <v>77</v>
@@ -1154,10 +1154,10 @@
         <v>74000</v>
       </c>
       <c r="H18" t="n">
-        <v>19.54280949797445</v>
+        <v>19.52695484553665</v>
       </c>
       <c r="I18" t="n">
-        <v>16.39201830240722</v>
+        <v>16.38224917302435</v>
       </c>
       <c r="J18" t="n">
         <v>105</v>
@@ -1226,7 +1226,7 @@
         <v>1400000</v>
       </c>
       <c r="H20" t="n">
-        <v>19.9401196371148</v>
+        <v>19.93945101197486</v>
       </c>
       <c r="J20" t="n">
         <v>81</v>
@@ -1259,10 +1259,10 @@
         <v>1204000</v>
       </c>
       <c r="H21" t="n">
-        <v>20.21847359340163</v>
+        <v>20.15445709110676</v>
       </c>
       <c r="I21" t="n">
-        <v>17.1860158326566</v>
+        <v>17.11781261270464</v>
       </c>
       <c r="J21" t="n">
         <v>176</v>
@@ -1295,7 +1295,7 @@
         <v>21320</v>
       </c>
       <c r="H22" t="n">
-        <v>20.41840307654648</v>
+        <v>20.41458137591642</v>
       </c>
       <c r="J22" t="n">
         <v>134</v>
@@ -1328,10 +1328,10 @@
         <v>114500</v>
       </c>
       <c r="H23" t="n">
-        <v>20.50315061539488</v>
+        <v>20.49242064997426</v>
       </c>
       <c r="I23" t="n">
-        <v>18.00406486584858</v>
+        <v>17.99470055418258</v>
       </c>
       <c r="J23" t="n">
         <v>96</v>
@@ -1364,10 +1364,10 @@
         <v>188111.1111111111</v>
       </c>
       <c r="H24" t="n">
-        <v>20.60852804622976</v>
+        <v>20.60035403289035</v>
       </c>
       <c r="I24" t="n">
-        <v>18.18708126735275</v>
+        <v>18.17996532532548</v>
       </c>
       <c r="J24" t="n">
         <v>115</v>
@@ -1400,10 +1400,10 @@
         <v>188111.1111111111</v>
       </c>
       <c r="H25" t="n">
-        <v>20.60852804622976</v>
+        <v>20.60035403289035</v>
       </c>
       <c r="I25" t="n">
-        <v>18.18708126735275</v>
+        <v>18.17996532532548</v>
       </c>
       <c r="J25" t="n">
         <v>195</v>
@@ -1436,10 +1436,10 @@
         <v>719032.2580645161</v>
       </c>
       <c r="H26" t="n">
-        <v>20.88392783136021</v>
+        <v>20.78271547037707</v>
       </c>
       <c r="I26" t="n">
-        <v>17.99953686425504</v>
+        <v>17.93177808701002</v>
       </c>
       <c r="J26" t="n">
         <v>177</v>
@@ -1472,7 +1472,7 @@
         <v>4.285714285714286</v>
       </c>
       <c r="H27" t="n">
-        <v>21.24285833888526</v>
+        <v>21.2401571660666</v>
       </c>
       <c r="J27" t="n">
         <v>67</v>
@@ -1505,10 +1505,10 @@
         <v>634888.8888888889</v>
       </c>
       <c r="H28" t="n">
-        <v>21.38162772523852</v>
+        <v>21.30442019260907</v>
       </c>
       <c r="I28" t="n">
-        <v>18.1658670688078</v>
+        <v>18.10680560829568</v>
       </c>
       <c r="J28" t="n">
         <v>82</v>
@@ -1541,10 +1541,10 @@
         <v>380000</v>
       </c>
       <c r="H29" t="n">
-        <v>21.48381139023793</v>
+        <v>21.37188136664816</v>
       </c>
       <c r="I29" t="n">
-        <v>18.18074192407538</v>
+        <v>18.09852931446574</v>
       </c>
       <c r="J29" t="n">
         <v>171</v>
@@ -1577,10 +1577,10 @@
         <v>73913.04347826086</v>
       </c>
       <c r="H30" t="n">
-        <v>21.52751642022882</v>
+        <v>21.52722858354669</v>
       </c>
       <c r="I30" t="n">
-        <v>18.22614320114317</v>
+        <v>18.22593428354077</v>
       </c>
       <c r="J30" t="n">
         <v>168</v>
@@ -1613,10 +1613,10 @@
         <v>81000</v>
       </c>
       <c r="H31" t="n">
-        <v>21.62045387520759</v>
+        <v>21.62004243546474</v>
       </c>
       <c r="I31" t="n">
-        <v>18.39789791214488</v>
+        <v>18.39761294088624</v>
       </c>
       <c r="J31" t="n">
         <v>169</v>
@@ -1649,10 +1649,10 @@
         <v>24038.46153846154</v>
       </c>
       <c r="H32" t="n">
-        <v>21.62982995673705</v>
+        <v>21.63012599814882</v>
       </c>
       <c r="I32" t="n">
-        <v>18.48106926843412</v>
+        <v>18.48118443757064</v>
       </c>
       <c r="J32" t="n">
         <v>117</v>
@@ -1685,10 +1685,10 @@
         <v>104000</v>
       </c>
       <c r="H33" t="n">
-        <v>21.64565328468139</v>
+        <v>21.64527485456869</v>
       </c>
       <c r="I33" t="n">
-        <v>18.41532748510019</v>
+        <v>18.41506608586634</v>
       </c>
       <c r="J33" t="n">
         <v>170</v>
@@ -1721,10 +1721,10 @@
         <v>2210833.333333333</v>
       </c>
       <c r="H34" t="n">
-        <v>21.72650615311951</v>
+        <v>21.76221947626512</v>
       </c>
       <c r="I34" t="n">
-        <v>18.8106786913261</v>
+        <v>18.8149928148991</v>
       </c>
       <c r="J34" t="n">
         <v>187</v>
@@ -1757,10 +1757,10 @@
         <v>38500</v>
       </c>
       <c r="H35" t="n">
-        <v>21.78946668425935</v>
+        <v>21.78930735776838</v>
       </c>
       <c r="I35" t="n">
-        <v>18.98122294877135</v>
+        <v>18.98098696378628</v>
       </c>
       <c r="J35" t="n">
         <v>167</v>
@@ -1793,10 +1793,10 @@
         <v>486000</v>
       </c>
       <c r="H36" t="n">
-        <v>21.92189577089803</v>
+        <v>21.92174435531882</v>
       </c>
       <c r="I36" t="n">
-        <v>19.29087967405975</v>
+        <v>19.29062764485845</v>
       </c>
       <c r="J36" t="n">
         <v>172</v>
@@ -1829,10 +1829,10 @@
         <v>144340</v>
       </c>
       <c r="H37" t="n">
-        <v>21.98558294896831</v>
+        <v>21.98536682360781</v>
       </c>
       <c r="I37" t="n">
-        <v>19.0056192911464</v>
+        <v>19.00547571699945</v>
       </c>
       <c r="J37" t="n">
         <v>175</v>
@@ -1865,10 +1865,10 @@
         <v>112220</v>
       </c>
       <c r="H38" t="n">
-        <v>22.10531417136249</v>
+        <v>22.10515879556368</v>
       </c>
       <c r="I38" t="n">
-        <v>19.08388631958708</v>
+        <v>19.08378650055852</v>
       </c>
       <c r="J38" t="n">
         <v>174</v>
@@ -1901,10 +1901,10 @@
         <v>95750</v>
       </c>
       <c r="H39" t="n">
-        <v>22.18403759214089</v>
+        <v>22.18328192693386</v>
       </c>
       <c r="I39" t="n">
-        <v>19.28895266215994</v>
+        <v>19.28841919428085</v>
       </c>
       <c r="J39" t="n">
         <v>178</v>
@@ -1937,10 +1937,10 @@
         <v>4146666.666666667</v>
       </c>
       <c r="H40" t="n">
-        <v>22.21762548777048</v>
+        <v>22.21693002558449</v>
       </c>
       <c r="I40" t="n">
-        <v>19.22613184874692</v>
+        <v>19.22566949948449</v>
       </c>
       <c r="J40" t="n">
         <v>190</v>
@@ -1973,10 +1973,10 @@
         <v>44480</v>
       </c>
       <c r="H41" t="n">
-        <v>22.24627089066778</v>
+        <v>22.23441804576935</v>
       </c>
       <c r="I41" t="n">
-        <v>18.39628638204979</v>
+        <v>18.38651705441137</v>
       </c>
       <c r="J41" t="n">
         <v>118</v>
@@ -2009,10 +2009,10 @@
         <v>1280000</v>
       </c>
       <c r="H42" t="n">
-        <v>22.30228578978384</v>
+        <v>22.26949764505553</v>
       </c>
       <c r="I42" t="n">
-        <v>19.73825180439047</v>
+        <v>19.71360341245012</v>
       </c>
       <c r="J42" t="n">
         <v>185</v>
@@ -2045,10 +2045,10 @@
         <v>342741.935483871</v>
       </c>
       <c r="H43" t="n">
-        <v>22.34666271419135</v>
+        <v>22.34629490641281</v>
       </c>
       <c r="I43" t="n">
-        <v>19.77671963556965</v>
+        <v>19.77644633535914</v>
       </c>
       <c r="J43" t="n">
         <v>101</v>
@@ -2081,10 +2081,10 @@
         <v>464250</v>
       </c>
       <c r="H44" t="n">
-        <v>22.40254117691718</v>
+        <v>22.401891205133</v>
       </c>
       <c r="I44" t="n">
-        <v>19.41929477239402</v>
+        <v>19.41897404157888</v>
       </c>
       <c r="J44" t="n">
         <v>180</v>
@@ -2117,10 +2117,10 @@
         <v>24000</v>
       </c>
       <c r="H45" t="n">
-        <v>22.4243867839569</v>
+        <v>22.42438620103372</v>
       </c>
       <c r="I45" t="n">
-        <v>20.26838805456152</v>
+        <v>20.2683867945907</v>
       </c>
       <c r="J45" t="n">
         <v>165</v>
@@ -2153,10 +2153,10 @@
         <v>5782608.695652174</v>
       </c>
       <c r="H46" t="n">
-        <v>22.43848613153626</v>
+        <v>22.43766932192126</v>
       </c>
       <c r="I46" t="n">
-        <v>19.9012117027526</v>
+        <v>19.90059826136212</v>
       </c>
       <c r="J46" t="n">
         <v>192</v>
@@ -2165,70 +2165,70 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>3.4 wt% Co–N–C</t>
+          <t>Ru/Pr2O3</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Co</t>
+          <t>Ru</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>3.73</v>
+        <v>5</v>
       </c>
       <c r="D47" t="n">
-        <v>350</v>
+        <v>400</v>
       </c>
       <c r="E47" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F47" t="n">
-        <v>4340</v>
+        <v>64000</v>
       </c>
       <c r="G47" t="n">
-        <v>116353.8873994638</v>
+        <v>1280000</v>
       </c>
       <c r="H47" t="n">
-        <v>22.54484973796892</v>
+        <v>22.50875227002852</v>
+      </c>
+      <c r="I47" t="n">
+        <v>19.11011498891022</v>
       </c>
       <c r="J47" t="n">
-        <v>200</v>
+        <v>182</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Ru/Pr2O3</t>
+          <t>3.4 wt% Co–N–C</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Ru</t>
+          <t>Co</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>5</v>
+        <v>3.73</v>
       </c>
       <c r="D48" t="n">
-        <v>400</v>
+        <v>350</v>
       </c>
       <c r="E48" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F48" t="n">
-        <v>64000</v>
+        <v>4340</v>
       </c>
       <c r="G48" t="n">
-        <v>1280000</v>
+        <v>116353.8873994638</v>
       </c>
       <c r="H48" t="n">
-        <v>22.58696610857199</v>
-      </c>
-      <c r="I48" t="n">
-        <v>19.18608642663893</v>
+        <v>22.54368102061514</v>
       </c>
       <c r="J48" t="n">
-        <v>182</v>
+        <v>200</v>
       </c>
     </row>
     <row r="49">
@@ -2258,10 +2258,10 @@
         <v>2240000</v>
       </c>
       <c r="H49" t="n">
-        <v>22.60674725199266</v>
+        <v>22.58972546066001</v>
       </c>
       <c r="I49" t="n">
-        <v>20.53557117927961</v>
+        <v>20.51610109982357</v>
       </c>
       <c r="J49" t="n">
         <v>184</v>
@@ -2294,10 +2294,10 @@
         <v>1080000</v>
       </c>
       <c r="H50" t="n">
-        <v>22.66155427079388</v>
+        <v>22.63422190250466</v>
       </c>
       <c r="I50" t="n">
-        <v>19.99958887695469</v>
+        <v>19.97839032758582</v>
       </c>
       <c r="J50" t="n">
         <v>186</v>
@@ -2330,10 +2330,10 @@
         <v>152500</v>
       </c>
       <c r="H51" t="n">
-        <v>22.73773953945267</v>
+        <v>22.73911866181321</v>
       </c>
       <c r="I51" t="n">
-        <v>20.06228377893208</v>
+        <v>20.06350601417598</v>
       </c>
       <c r="J51" t="n">
         <v>162</v>
@@ -2366,10 +2366,10 @@
         <v>2106666.666666667</v>
       </c>
       <c r="H52" t="n">
-        <v>22.79787449624272</v>
+        <v>22.79707615469821</v>
       </c>
       <c r="I52" t="n">
-        <v>19.67159306583043</v>
+        <v>19.67121736144116</v>
       </c>
       <c r="J52" t="n">
         <v>191</v>
@@ -2402,10 +2402,10 @@
         <v>3279069.76744186</v>
       </c>
       <c r="H53" t="n">
-        <v>22.97770863250099</v>
+        <v>22.97505023442373</v>
       </c>
       <c r="I53" t="n">
-        <v>21.14159159296535</v>
+        <v>21.13842463633245</v>
       </c>
       <c r="J53" t="n">
         <v>81</v>
@@ -2438,7 +2438,7 @@
         <v>67.22689075630252</v>
       </c>
       <c r="H54" t="n">
-        <v>23.08299364512096</v>
+        <v>23.08299349565035</v>
       </c>
       <c r="J54" t="n">
         <v>76</v>
@@ -2471,10 +2471,10 @@
         <v>215000</v>
       </c>
       <c r="H55" t="n">
-        <v>23.20513240513247</v>
+        <v>23.20436073707794</v>
       </c>
       <c r="I55" t="n">
-        <v>20.12113185576782</v>
+        <v>20.12072416313562</v>
       </c>
       <c r="J55" t="n">
         <v>181</v>
@@ -2507,10 +2507,10 @@
         <v>181500</v>
       </c>
       <c r="H56" t="n">
-        <v>23.21754723436856</v>
+        <v>23.22687763512296</v>
       </c>
       <c r="I56" t="n">
-        <v>20.46191590280913</v>
+        <v>20.46935647932307</v>
       </c>
       <c r="J56" t="n">
         <v>164</v>
@@ -2543,10 +2543,10 @@
         <v>32225</v>
       </c>
       <c r="H57" t="n">
-        <v>23.22789996923463</v>
+        <v>23.22776998802789</v>
       </c>
       <c r="I57" t="n">
-        <v>19.81693600574157</v>
+        <v>19.81687091043289</v>
       </c>
       <c r="J57" t="n">
         <v>178</v>
@@ -2579,10 +2579,10 @@
         <v>210000</v>
       </c>
       <c r="H58" t="n">
-        <v>23.30663036319694</v>
+        <v>23.30580558092457</v>
       </c>
       <c r="I58" t="n">
-        <v>20.68915510023711</v>
+        <v>20.68866835664272</v>
       </c>
       <c r="J58" t="n">
         <v>179</v>
@@ -2615,10 +2615,10 @@
         <v>391750</v>
       </c>
       <c r="H59" t="n">
-        <v>23.32994138420145</v>
+        <v>23.32917066895267</v>
       </c>
       <c r="I59" t="n">
-        <v>19.86733676694525</v>
+        <v>19.86696646925644</v>
       </c>
       <c r="J59" t="n">
         <v>94</v>
@@ -2651,10 +2651,10 @@
         <v>418701.2987012987</v>
       </c>
       <c r="H60" t="n">
-        <v>23.3806887186201</v>
+        <v>23.37988813206525</v>
       </c>
       <c r="I60" t="n">
-        <v>19.93166290933067</v>
+        <v>19.93127182313833</v>
       </c>
       <c r="J60" t="n">
         <v>183</v>
@@ -2687,10 +2687,10 @@
         <v>382383.4196891192</v>
       </c>
       <c r="H61" t="n">
-        <v>23.49981359461895</v>
+        <v>23.49895488665815</v>
       </c>
       <c r="I61" t="n">
-        <v>19.98685282787688</v>
+        <v>19.98643144807416</v>
       </c>
       <c r="J61" t="n">
         <v>183</v>
@@ -2723,10 +2723,10 @@
         <v>960000</v>
       </c>
       <c r="H62" t="n">
-        <v>23.54534376164739</v>
+        <v>23.51767409881526</v>
       </c>
       <c r="I62" t="n">
-        <v>20.52873756182436</v>
+        <v>20.51356024600929</v>
       </c>
       <c r="J62" t="n">
         <v>188</v>
@@ -2759,7 +2759,7 @@
         <v>240</v>
       </c>
       <c r="H63" t="n">
-        <v>23.71054962146314</v>
+        <v>23.71054935914687</v>
       </c>
       <c r="J63" t="n">
         <v>79</v>
@@ -2792,10 +2792,10 @@
         <v>1410000</v>
       </c>
       <c r="H64" t="n">
-        <v>23.71111091493324</v>
+        <v>23.7109326477648</v>
       </c>
       <c r="I64" t="n">
-        <v>22.46339128522992</v>
+        <v>22.4632665502814</v>
       </c>
       <c r="J64" t="n">
         <v>173</v>
@@ -2828,7 +2828,7 @@
         <v>860000</v>
       </c>
       <c r="H65" t="n">
-        <v>23.7370653751148</v>
+        <v>23.73387896628061</v>
       </c>
       <c r="J65" t="n">
         <v>206</v>
@@ -2861,7 +2861,7 @@
         <v>16400</v>
       </c>
       <c r="H66" t="n">
-        <v>24.08428688319593</v>
+        <v>24.08394547182962</v>
       </c>
       <c r="J66" t="n">
         <v>134</v>
@@ -2894,10 +2894,10 @@
         <v>184750</v>
       </c>
       <c r="H67" t="n">
-        <v>24.4107382267625</v>
+        <v>24.41007009522229</v>
       </c>
       <c r="I67" t="n">
-        <v>20.40037538048987</v>
+        <v>20.39998074223815</v>
       </c>
       <c r="J67" t="n">
         <v>94</v>
@@ -2930,10 +2930,10 @@
         <v>200000</v>
       </c>
       <c r="H68" t="n">
-        <v>24.71430488603433</v>
+        <v>24.80386642961499</v>
       </c>
       <c r="I68" t="n">
-        <v>21.66668781140656</v>
+        <v>21.73392142828638</v>
       </c>
       <c r="J68" t="n">
         <v>164</v>
@@ -2966,10 +2966,10 @@
         <v>3235294.117647059</v>
       </c>
       <c r="H69" t="n">
-        <v>24.90675306015482</v>
+        <v>24.9059971986012</v>
       </c>
       <c r="I69" t="n">
-        <v>20.89006273912438</v>
+        <v>20.88959536260946</v>
       </c>
       <c r="J69" t="n">
         <v>194</v>
@@ -2978,70 +2978,70 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Ru/C12A7 (microcube)</t>
+          <t>NI/CeN NPs</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Ru</t>
+          <t>Ni</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>5</v>
+        <v>11.7</v>
       </c>
       <c r="D70" t="n">
         <v>400</v>
       </c>
       <c r="E70" t="n">
-        <v>0.1</v>
+        <v>0.9</v>
       </c>
       <c r="F70" t="n">
-        <v>5380</v>
+        <v>6500</v>
       </c>
       <c r="G70" t="n">
-        <v>107600</v>
+        <v>55555.55555555556</v>
       </c>
       <c r="H70" t="n">
-        <v>25.45190220769257</v>
-      </c>
-      <c r="I70" t="n">
-        <v>21.4021461193574</v>
+        <v>25.9193907089895</v>
       </c>
       <c r="J70" t="n">
-        <v>196</v>
+        <v>150</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>NI/CeN NPs</t>
+          <t>Ru/C12A7 (microcube)</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Ni</t>
+          <t>Ru</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>11.7</v>
+        <v>5</v>
       </c>
       <c r="D71" t="n">
         <v>400</v>
       </c>
       <c r="E71" t="n">
-        <v>0.9</v>
+        <v>0.1</v>
       </c>
       <c r="F71" t="n">
-        <v>6500</v>
+        <v>5380</v>
       </c>
       <c r="G71" t="n">
-        <v>55555.55555555556</v>
+        <v>107600</v>
       </c>
       <c r="H71" t="n">
-        <v>25.92523059474333</v>
+        <v>26.20136441171531</v>
+      </c>
+      <c r="I71" t="n">
+        <v>21.9371504230411</v>
       </c>
       <c r="J71" t="n">
-        <v>150</v>
+        <v>196</v>
       </c>
     </row>
     <row r="72">
@@ -3071,10 +3071,10 @@
         <v>514629.6296296296</v>
       </c>
       <c r="H72" t="n">
-        <v>26.72546206061724</v>
+        <v>26.717317081552</v>
       </c>
       <c r="I72" t="n">
-        <v>25.12452229978249</v>
+        <v>25.11588950800139</v>
       </c>
       <c r="J72" t="n">
         <v>163</v>
@@ -3083,70 +3083,70 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>6 wt% Co/CeO2</t>
+          <t>Ru/CeO2-r</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Co</t>
+          <t>Ru</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D73" t="n">
-        <v>430</v>
+        <v>400</v>
       </c>
       <c r="E73" t="n">
         <v>10</v>
       </c>
       <c r="F73" t="n">
-        <v>26654</v>
+        <v>115000</v>
       </c>
       <c r="G73" t="n">
-        <v>444233.3333333334</v>
+        <v>1150000</v>
       </c>
       <c r="H73" t="n">
-        <v>28.15030177609778</v>
+        <v>28.11549732185807</v>
+      </c>
+      <c r="I73" t="n">
+        <v>22.80727609747251</v>
       </c>
       <c r="J73" t="n">
-        <v>205</v>
+        <v>100</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Ru/CeO2-r</t>
+          <t>6 wt% Co/CeO2</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Ru</t>
+          <t>Co</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D74" t="n">
-        <v>400</v>
+        <v>430</v>
       </c>
       <c r="E74" t="n">
         <v>10</v>
       </c>
       <c r="F74" t="n">
-        <v>115000</v>
+        <v>26654</v>
       </c>
       <c r="G74" t="n">
-        <v>1150000</v>
+        <v>444233.3333333334</v>
       </c>
       <c r="H74" t="n">
-        <v>28.16239364178105</v>
-      </c>
-      <c r="I74" t="n">
-        <v>22.83375809565127</v>
+        <v>28.14354075398602</v>
       </c>
       <c r="J74" t="n">
-        <v>100</v>
+        <v>205</v>
       </c>
     </row>
     <row r="75">
@@ -3176,7 +3176,7 @@
         <v>67846.15384615384</v>
       </c>
       <c r="H75" t="n">
-        <v>35.15353985646534</v>
+        <v>35.13257848346144</v>
       </c>
       <c r="J75" t="n">
         <v>197</v>
@@ -3209,10 +3209,10 @@
         <v>9750</v>
       </c>
       <c r="H76" t="n">
-        <v>41.27808885912891</v>
+        <v>41.27598549929062</v>
       </c>
       <c r="I76" t="n">
-        <v>30.31078449179117</v>
+        <v>30.30968171443131</v>
       </c>
       <c r="J76" t="n">
         <v>94</v>
@@ -3273,7 +3273,7 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>17.52559198205939</v>
+        <v>17.22165142925473</v>
       </c>
     </row>
     <row r="85">
@@ -3305,7 +3305,7 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>0.1443268610664097</v>
+        <v>0.1244811783015827</v>
       </c>
     </row>
     <row r="88">
@@ -3315,7 +3315,7 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>0.1562871203122349</v>
+        <v>0.1582000215972726</v>
       </c>
     </row>
   </sheetData>
@@ -3429,7 +3429,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>15.51555967209343</v>
+        <v>15.5091508671665</v>
       </c>
       <c r="D5" t="n">
         <v>9</v>
@@ -3447,7 +3447,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>18.27959353487723</v>
+        <v>18.27631008120813</v>
       </c>
       <c r="D6" t="n">
         <v>5</v>
@@ -3465,7 +3465,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>20.41840307654648</v>
+        <v>20.41458137591642</v>
       </c>
       <c r="D7" t="n">
         <v>5</v>

</xml_diff>